<commit_message>
CG0253 create: attempt to use variable is null operation
</commit_message>
<xml_diff>
--- a/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
+++ b/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marisa_wyckmans\CORE\CDISC_Rule_Authoring\core-contributor\rules\NEW-RULE\negative\01\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC156351-921E-46C5-B037-B0AC2D3B5CDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0CB2333-E90C-4BFC-A837-01C91720BEC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="21240" windowHeight="15270" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,20 @@
     <sheet name="Validation" sheetId="3" r:id="rId3"/>
     <sheet name="ti.xpt" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -215,7 +228,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -227,9 +240,6 @@
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -709,7 +719,7 @@
         <v>12</v>
       </c>
       <c r="C4" t="s">
-        <v>37</v>
+        <v>10</v>
       </c>
       <c r="D4">
         <v>5</v>
@@ -786,7 +796,7 @@
         <v>12</v>
       </c>
       <c r="C8" t="s">
-        <v>37</v>
+        <v>10</v>
       </c>
       <c r="D8">
         <v>7</v>
@@ -912,7 +922,7 @@
       <c r="A5" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="3" t="s">
         <v>28</v>
       </c>
       <c r="C5" s="4" t="s">
@@ -921,7 +931,7 @@
       <c r="D5" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="3" t="s">
         <v>31</v>
       </c>
       <c r="F5" s="4"/>
@@ -930,25 +940,24 @@
       <c r="A6" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="E6" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="F6" s="5"/>
     </row>
     <row r="7" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="3" t="s">
         <v>28</v>
       </c>
       <c r="C7" s="4" t="s">
@@ -957,7 +966,7 @@
       <c r="D7" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="E7" s="3" t="s">
         <v>31</v>
       </c>
       <c r="F7" s="4"/>

</xml_diff>

<commit_message>
CG0012 create / CORE-001082 edit: test data updated and rule fully validated
</commit_message>
<xml_diff>
--- a/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
+++ b/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marisa_wyckmans\CORE\CDISC_Rule_Authoring\core-contributor\rules\NEW-RULE\negative\01\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{262B1228-DA4C-4C4E-AAB2-D0DCC6F22BAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8B605B8-9A1F-4C81-A7A6-77F6D4981C35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="21240" windowHeight="15270" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="1" r:id="rId1"/>
@@ -403,7 +403,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -442,20 +442,8 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
   </fonts>
-  <fills count="8">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -464,33 +452,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
+        <fgColor rgb="FFFFFFCC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFCC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -506,19 +473,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1311,7 +1274,7 @@
       <c r="E20" t="s">
         <v>18</v>
       </c>
-      <c r="F20" s="11" t="s">
+      <c r="F20" s="5" t="s">
         <v>114</v>
       </c>
     </row>
@@ -1331,7 +1294,7 @@
       <c r="E21" t="s">
         <v>20</v>
       </c>
-      <c r="F21" s="11" t="s">
+      <c r="F21" s="5" t="s">
         <v>23</v>
       </c>
     </row>
@@ -1348,7 +1311,7 @@
       <c r="E22" t="s">
         <v>22</v>
       </c>
-      <c r="F22" s="11" t="s">
+      <c r="F22" s="5" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1368,7 +1331,7 @@
       <c r="E23" t="s">
         <v>18</v>
       </c>
-      <c r="F23" s="11" t="s">
+      <c r="F23" s="5" t="s">
         <v>120</v>
       </c>
     </row>
@@ -1388,7 +1351,7 @@
       <c r="E24" t="s">
         <v>20</v>
       </c>
-      <c r="F24" s="11" t="s">
+      <c r="F24" s="5" t="s">
         <v>23</v>
       </c>
     </row>
@@ -1405,7 +1368,7 @@
       <c r="E25" t="s">
         <v>22</v>
       </c>
-      <c r="F25" s="11" t="s">
+      <c r="F25" s="5" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1427,274 +1390,274 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="I1" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="J1" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="K1" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="L1" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="M1" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="N1" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="O1" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="P1" s="3" t="s">
+      <c r="P1" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="Q1" s="3" t="s">
+      <c r="Q1" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="R1" s="3" t="s">
+      <c r="R1" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="S1" s="3" t="s">
+      <c r="S1" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="T1" s="3" t="s">
+      <c r="T1" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="U1" s="3" t="s">
+      <c r="U1" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="V1" s="9" t="s">
+      <c r="V1" s="7" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="G2" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="H2" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="I2" s="4" t="s">
+      <c r="I2" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="J2" s="4" t="s">
+      <c r="J2" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="K2" s="4" t="s">
+      <c r="K2" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="L2" s="4" t="s">
+      <c r="L2" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="M2" s="4" t="s">
+      <c r="M2" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="N2" s="4" t="s">
+      <c r="N2" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="O2" s="4" t="s">
+      <c r="O2" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="P2" s="4" t="s">
+      <c r="P2" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="Q2" s="4" t="s">
+      <c r="Q2" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="R2" s="4" t="s">
+      <c r="R2" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="S2" s="4" t="s">
+      <c r="S2" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="T2" s="4" t="s">
+      <c r="T2" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="U2" s="4" t="s">
+      <c r="U2" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="V2" s="4" t="s">
+      <c r="V2" s="3" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="3" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="G3" s="8" t="s">
+      <c r="B3" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G3" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="H3" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="I3" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="J3" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="K3" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="L3" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="M3" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="N3" s="4" t="s">
+      <c r="H3" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="L3" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="M3" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="N3" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="O3" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="P3" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="Q3" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="R3" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="S3" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="T3" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="U3" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="V3" s="8" t="s">
+      <c r="O3" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="P3" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q3" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="R3" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="S3" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="T3" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="U3" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="V3" s="3" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A4" s="4">
+      <c r="A4" s="3">
         <v>10</v>
       </c>
-      <c r="B4" s="4">
+      <c r="B4" s="3">
         <v>2</v>
       </c>
-      <c r="C4" s="4">
+      <c r="C4" s="3">
         <v>14</v>
       </c>
-      <c r="D4" s="4">
+      <c r="D4" s="3">
         <v>3</v>
       </c>
-      <c r="E4" s="4">
+      <c r="E4" s="3">
         <v>10</v>
       </c>
-      <c r="F4" s="4">
+      <c r="F4" s="3">
         <v>10</v>
       </c>
-      <c r="G4" s="4">
+      <c r="G4" s="3">
         <v>10</v>
       </c>
-      <c r="H4" s="4">
+      <c r="H4" s="3">
         <v>10</v>
       </c>
-      <c r="I4" s="4">
+      <c r="I4" s="3">
         <v>10</v>
       </c>
-      <c r="J4" s="4">
+      <c r="J4" s="3">
         <v>10</v>
       </c>
-      <c r="K4" s="4">
+      <c r="K4" s="3">
         <v>1</v>
       </c>
-      <c r="L4" s="4">
+      <c r="L4" s="3">
         <v>1</v>
       </c>
-      <c r="M4" s="4">
+      <c r="M4" s="3">
         <v>3</v>
       </c>
-      <c r="N4" s="4">
+      <c r="N4" s="3">
         <v>8</v>
       </c>
-      <c r="O4" s="4">
+      <c r="O4" s="3">
         <v>5</v>
       </c>
-      <c r="P4" s="4">
+      <c r="P4" s="3">
         <v>1</v>
       </c>
-      <c r="Q4" s="4">
+      <c r="Q4" s="3">
         <v>1</v>
       </c>
-      <c r="R4" s="4">
+      <c r="R4" s="3">
         <v>1</v>
       </c>
-      <c r="S4" s="4">
+      <c r="S4" s="3">
         <v>13</v>
       </c>
-      <c r="T4" s="4">
+      <c r="T4" s="3">
         <v>1</v>
       </c>
-      <c r="U4" s="4">
+      <c r="U4" s="3">
         <v>13</v>
       </c>
-      <c r="V4" s="4">
+      <c r="V4" s="3">
         <v>3</v>
       </c>
     </row>
@@ -1780,178 +1743,178 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="J1" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="K1" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="L1" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="M1" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="N1" s="6" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="G2" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="H2" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="I2" s="4" t="s">
+      <c r="I2" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="J2" s="4" t="s">
+      <c r="J2" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="K2" s="4" t="s">
+      <c r="K2" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="L2" s="4" t="s">
+      <c r="L2" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="M2" s="4" t="s">
+      <c r="M2" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="N2" s="4" t="s">
+      <c r="N2" s="3" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="D3" s="4" t="s">
+      <c r="A3" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="E3" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="G3" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="H3" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="I3" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="J3" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="K3" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="L3" s="4" t="s">
+      <c r="E3" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="L3" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="M3" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="N3" s="8" t="s">
+      <c r="M3" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="N3" s="3" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A4" s="4">
+      <c r="A4" s="3">
         <v>10</v>
       </c>
-      <c r="B4" s="4">
+      <c r="B4" s="3">
         <v>2</v>
       </c>
-      <c r="C4" s="4">
+      <c r="C4" s="3">
         <v>14</v>
       </c>
-      <c r="D4" s="4">
+      <c r="D4" s="3">
         <v>8</v>
       </c>
-      <c r="E4" s="4">
+      <c r="E4" s="3">
         <v>8</v>
       </c>
-      <c r="F4" s="4">
+      <c r="F4" s="3">
         <v>40</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="G4" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="H4" s="4" t="s">
+      <c r="H4" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="I4" s="4">
+      <c r="I4" s="3">
         <v>8</v>
       </c>
-      <c r="J4" s="4">
+      <c r="J4" s="3">
         <v>18</v>
       </c>
-      <c r="K4" s="4">
+      <c r="K4" s="3">
         <v>10</v>
       </c>
-      <c r="L4" s="4">
+      <c r="L4" s="3">
         <v>8</v>
       </c>
-      <c r="M4" s="4">
+      <c r="M4" s="3">
         <v>8</v>
       </c>
-      <c r="N4" s="4" t="s">
+      <c r="N4" s="3" t="s">
         <v>104</v>
       </c>
     </row>
@@ -2013,154 +1976,154 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="I1" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="J1" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="K1" s="7" t="s">
         <v>119</v>
       </c>
-      <c r="L1" s="9" t="s">
+      <c r="L1" s="7" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="F2" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="G2" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="H2" s="6" t="s">
+      <c r="H2" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="I2" s="6" t="s">
+      <c r="I2" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="J2" s="6" t="s">
+      <c r="J2" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="K2" s="6" t="s">
+      <c r="K2" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="L2" s="6" t="s">
+      <c r="L2" s="4" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A3" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="D3" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="E3" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="F3" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="G3" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="H3" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="I3" s="6" t="s">
+      <c r="A3" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="I3" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="J3" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="K3" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L3" s="10" t="s">
+      <c r="J3" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="K3" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="L3" s="4" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A4" s="6">
+      <c r="A4" s="4">
         <v>10</v>
       </c>
-      <c r="B4" s="6">
+      <c r="B4" s="4">
         <v>2</v>
       </c>
-      <c r="C4" s="6">
+      <c r="C4" s="4">
         <v>14</v>
       </c>
-      <c r="D4" s="6">
+      <c r="D4" s="4">
         <v>8</v>
       </c>
-      <c r="E4" s="6">
+      <c r="E4" s="4">
         <v>8</v>
       </c>
-      <c r="F4" s="6">
+      <c r="F4" s="4">
         <v>40</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="G4" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="H4" s="6" t="s">
+      <c r="H4" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="I4" s="6">
+      <c r="I4" s="4">
         <v>8</v>
       </c>
-      <c r="J4" s="6">
+      <c r="J4" s="4">
         <v>18</v>
       </c>
-      <c r="K4" s="6">
+      <c r="K4" s="4">
         <v>10</v>
       </c>
-      <c r="L4" s="6">
+      <c r="L4" s="4">
         <v>8</v>
       </c>
     </row>

</xml_diff>

<commit_message>
created rule CG0651, test data and ran a validation
</commit_message>
<xml_diff>
--- a/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
+++ b/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
@@ -1,19 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\els_janssens\CORE\Rule_Authoring\core-contributor\rules\NEW-RULE\negative\01\data\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{980110FD-4C66-4324-868E-B291468F758E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="2"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet r:id="rId1" sheetId="1" name="Library"/>
-    <sheet r:id="rId2" sheetId="2" name="Datasets"/>
-    <sheet r:id="rId3" sheetId="3" name="Validation"/>
-    <sheet r:id="rId4" sheetId="4" name="sv.xpt"/>
-    <sheet r:id="rId5" sheetId="5" name="tv.xpt"/>
+    <sheet name="Library" sheetId="1" r:id="rId1"/>
+    <sheet name="Datasets" sheetId="2" r:id="rId2"/>
+    <sheet name="Validation" sheetId="3" r:id="rId3"/>
+    <sheet name="sv.xpt" sheetId="4" r:id="rId4"/>
+    <sheet name="tv.xpt" sheetId="5" r:id="rId5"/>
   </sheets>
-  <calcPr fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -254,9 +260,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
-  <numFmts count="0"/>
-  <fonts count="5" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -290,6 +295,14 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -300,7 +313,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFffffcc"/>
+        <fgColor rgb="FFFFFFCC"/>
       </patternFill>
     </fill>
   </fills>
@@ -321,16 +334,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FFc6c6c6"/>
+        <color rgb="FFC6C6C6"/>
       </left>
       <right style="thin">
-        <color rgb="FFc6c6c6"/>
+        <color rgb="FFC6C6C6"/>
       </right>
       <top style="thin">
-        <color rgb="FFc6c6c6"/>
+        <color rgb="FFC6C6C6"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFc6c6c6"/>
+        <color rgb="FFC6C6C6"/>
       </bottom>
       <diagonal/>
     </border>
@@ -338,56 +351,52 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+  <cellXfs count="13">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="2" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="2" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" builtinId="0" name="Normal"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -398,10 +407,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr lastClr="000000" val="windowText"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr lastClr="FFFFFF" val="window"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="1F497D"/>
@@ -439,71 +448,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Times New Roman" script="Arab"/>
-        <a:font typeface="Times New Roman" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="MoolBoran" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Times New Roman" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Arial" script="Arab"/>
-        <a:font typeface="Arial" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="DaunPenh" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Arial" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -531,7 +540,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -554,11 +563,11 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="9500"/>
@@ -567,13 +576,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -583,7 +592,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -592,7 +601,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -601,7 +610,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -609,10 +618,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot rev="0" lon="0" lat="0"/>
+              <a:rot lat="0" lon="0" rev="0"/>
             </a:camera>
-            <a:lightRig dir="t" rig="threePt">
-              <a:rot rev="1200000" lon="0" lat="0"/>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -677,18 +686,17 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="2" width="13.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
         <v>73</v>
       </c>
@@ -696,7 +704,7 @@
         <v>74</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+    <row r="2" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
         <v>75</v>
       </c>
@@ -710,18 +718,17 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="2" width="13.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
         <v>69</v>
       </c>
@@ -729,7 +736,7 @@
         <v>70</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+    <row r="2" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
         <v>58</v>
       </c>
@@ -737,7 +744,7 @@
         <v>71</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+    <row r="3" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>67</v>
       </c>
@@ -751,43 +758,43 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:F9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="13" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="9" width="49.14785714285715" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="10.85546875" style="9" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="27.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
-      <c r="A1" s="10" t="s">
+    <row r="1" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="12" t="s">
         <v>53</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="12" t="s">
         <v>54</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="F1" s="11" t="s">
+      <c r="F1" s="12" t="s">
         <v>57</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
-      <c r="A2" s="12">
+    <row r="2" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="10">
         <v>1</v>
       </c>
       <c r="B2" s="7" t="s">
@@ -806,8 +813,8 @@
         <v>3</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
-      <c r="A3" s="12">
+    <row r="3" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="10">
         <v>1</v>
       </c>
       <c r="B3" s="7" t="s">
@@ -826,8 +833,8 @@
         <v>62</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
-      <c r="A4" s="12">
+    <row r="4" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="10">
         <v>1</v>
       </c>
       <c r="B4" s="7" t="s">
@@ -846,8 +853,8 @@
         <v>64</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
-      <c r="A5" s="12">
+    <row r="5" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="10">
         <v>1</v>
       </c>
       <c r="B5" s="7" t="s">
@@ -866,8 +873,8 @@
         <v>66</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
-      <c r="A6" s="12">
+    <row r="6" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="10">
         <v>2</v>
       </c>
       <c r="B6" s="7" t="s">
@@ -886,8 +893,8 @@
         <v>68</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
-      <c r="A7" s="12">
+    <row r="7" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="10">
         <v>2</v>
       </c>
       <c r="B7" s="7" t="s">
@@ -906,8 +913,8 @@
         <v>62</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
-      <c r="A8" s="12">
+    <row r="8" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="10">
         <v>2</v>
       </c>
       <c r="B8" s="7" t="s">
@@ -926,8 +933,8 @@
         <v>64</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
-      <c r="A9" s="12">
+    <row r="9" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="10">
         <v>2</v>
       </c>
       <c r="B9" s="7" t="s">
@@ -952,27 +959,19 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:K7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="2" width="13.5703125" style="8" bestFit="1" customWidth="1"/>
+    <col min="3" max="6" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="11" width="13.5703125" style="8" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+    <row r="1" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1007,7 +1006,7 @@
         <v>35</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+    <row r="2" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>6</v>
       </c>
@@ -1042,7 +1041,7 @@
         <v>43</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+    <row r="3" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>12</v>
       </c>
@@ -1077,7 +1076,7 @@
         <v>12</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+    <row r="4" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5">
         <v>12</v>
       </c>
@@ -1112,7 +1111,7 @@
         <v>30</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
+    <row r="5" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>18</v>
       </c>
@@ -1143,7 +1142,7 @@
       <c r="J5" s="6"/>
       <c r="K5" s="6"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
+    <row r="6" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>18</v>
       </c>
@@ -1174,7 +1173,7 @@
       <c r="J6" s="6"/>
       <c r="K6" s="6"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
+    <row r="7" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>18</v>
       </c>
@@ -1211,22 +1210,18 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:F8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="2" width="13.5703125" style="8" bestFit="1" customWidth="1"/>
+    <col min="3" max="6" width="13.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+    <row r="1" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1246,7 +1241,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+    <row r="2" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>6</v>
       </c>
@@ -1266,7 +1261,7 @@
         <v>11</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+    <row r="3" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>12</v>
       </c>
@@ -1286,7 +1281,7 @@
         <v>12</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+    <row r="4" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5">
         <v>12</v>
       </c>
@@ -1306,7 +1301,7 @@
         <v>17</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
+    <row r="5" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>18</v>
       </c>
@@ -1324,7 +1319,7 @@
         <v>21</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
+    <row r="6" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>18</v>
       </c>
@@ -1340,7 +1335,7 @@
         <v>23</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
+    <row r="7" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>18</v>
       </c>
@@ -1358,7 +1353,7 @@
         <v>25</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
+    <row r="8" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
         <v>18</v>
       </c>

</xml_diff>

<commit_message>
CG0253 create: rule created based on info in GitHub Transfer Excel Tracker
</commit_message>
<xml_diff>
--- a/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
+++ b/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marisa_wyckmans\CORE\CDISC_Rule_Authoring\core-contributor\rules\NEW-RULE\negative\01\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D1184AB-5327-4B3F-BB6B-7E20A16B74EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28A6BE34-48B0-4334-ACFD-05C2572342D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="38">
   <si>
     <t>Product</t>
   </si>
@@ -150,12 +150,6 @@
   </si>
   <si>
     <t>Record</t>
-  </si>
-  <si>
-    <t>$record_count_ietestcd_ietest</t>
-  </si>
-  <si>
-    <t>$max_record_count_ietestcd_ietest</t>
   </si>
 </sst>
 </file>
@@ -647,7 +641,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="5" max="5" width="28.5703125" bestFit="1" customWidth="1"/>
@@ -694,7 +688,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
@@ -708,10 +702,7 @@
         <v>5</v>
       </c>
       <c r="E3" t="s">
-        <v>17</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>30</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -725,10 +716,13 @@
         <v>37</v>
       </c>
       <c r="D4">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E4" t="s">
-        <v>19</v>
+        <v>16</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -742,18 +736,15 @@
         <v>37</v>
       </c>
       <c r="D5">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E5" t="s">
-        <v>38</v>
-      </c>
-      <c r="F5">
-        <v>2</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B6" t="s">
         <v>12</v>
@@ -762,18 +753,18 @@
         <v>37</v>
       </c>
       <c r="D6">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E6" t="s">
-        <v>39</v>
-      </c>
-      <c r="F6">
-        <v>2</v>
+        <v>16</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B7" t="s">
         <v>12</v>
@@ -782,18 +773,15 @@
         <v>37</v>
       </c>
       <c r="D7">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E7" t="s">
-        <v>16</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B8" t="s">
         <v>12</v>
@@ -802,18 +790,18 @@
         <v>37</v>
       </c>
       <c r="D8">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E8" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B9" t="s">
         <v>12</v>
@@ -822,50 +810,10 @@
         <v>37</v>
       </c>
       <c r="D9">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E9" t="s">
         <v>19</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10">
-        <v>1</v>
-      </c>
-      <c r="B10" t="s">
-        <v>12</v>
-      </c>
-      <c r="C10" t="s">
-        <v>37</v>
-      </c>
-      <c r="D10">
-        <v>7</v>
-      </c>
-      <c r="E10" t="s">
-        <v>38</v>
-      </c>
-      <c r="F10">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11">
-        <v>1</v>
-      </c>
-      <c r="B11" t="s">
-        <v>12</v>
-      </c>
-      <c r="C11" t="s">
-        <v>37</v>
-      </c>
-      <c r="D11">
-        <v>7</v>
-      </c>
-      <c r="E11" t="s">
-        <v>39</v>
-      </c>
-      <c r="F11">
-        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -971,7 +919,7 @@
       <c r="C5" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="3" t="s">
         <v>30</v>
       </c>
       <c r="E5" s="3" t="s">
@@ -986,7 +934,7 @@
       <c r="B6" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="4" t="s">
         <v>33</v>
       </c>
       <c r="D6" s="3" t="s">
@@ -995,6 +943,7 @@
       <c r="E6" s="3" t="s">
         <v>32</v>
       </c>
+      <c r="F6" s="4"/>
     </row>
     <row r="7" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
@@ -1006,7 +955,7 @@
       <c r="C7" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="3" t="s">
         <v>30</v>
       </c>
       <c r="E7" s="3" t="s">
@@ -1021,7 +970,7 @@
       <c r="B8" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="4" t="s">
         <v>35</v>
       </c>
       <c r="D8" s="3" t="s">
@@ -1030,6 +979,7 @@
       <c r="E8" s="3" t="s">
         <v>32</v>
       </c>
+      <c r="F8" s="4"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:G4">

</xml_diff>

<commit_message>
CG0011 create: Part C rule created and tested
</commit_message>
<xml_diff>
--- a/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
+++ b/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marisa_wyckmans\CORE\CDISC_Rule_Authoring\core-contributor\rules\NEW-RULE\negative\01\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFB81727-433B-4851-954F-3F05AD7667EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{263E4ADE-82B5-4F59-B687-709514A24A27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="555" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-19310" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="377" uniqueCount="141">
   <si>
     <t>Product</t>
   </si>
@@ -442,6 +442,12 @@
   </si>
   <si>
     <t>TD</t>
+  </si>
+  <si>
+    <t>variable_value</t>
+  </si>
+  <si>
+    <t>variable_name</t>
   </si>
 </sst>
 </file>
@@ -482,7 +488,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -499,6 +505,12 @@
         <fgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -512,7 +524,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -530,6 +542,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -944,7 +957,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="5" max="5" width="14.28515625" bestFit="1" customWidth="1"/>
@@ -979,21 +992,21 @@
         <v>6</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D2">
-        <v>8</v>
-      </c>
-      <c r="E2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E2" t="s">
+        <v>140</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>19</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>6</v>
@@ -1002,38 +1015,38 @@
         <v>18</v>
       </c>
       <c r="D3">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E3" t="s">
-        <v>21</v>
-      </c>
-      <c r="F3" t="s">
-        <v>22</v>
+        <v>139</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D4">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E4" t="s">
-        <v>23</v>
+        <v>140</v>
       </c>
       <c r="F4" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>6</v>
@@ -1042,180 +1055,417 @@
         <v>18</v>
       </c>
       <c r="D5">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E5" t="s">
-        <v>25</v>
+        <v>139</v>
       </c>
       <c r="F5" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D6">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="E6" t="s">
-        <v>27</v>
+        <v>140</v>
       </c>
       <c r="F6" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7">
+        <v>3</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>6</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>8</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D7" s="1">
-        <v>5</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>22</v>
+      <c r="D7">
+        <v>6</v>
+      </c>
+      <c r="E7" t="s">
+        <v>139</v>
+      </c>
+      <c r="F7" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D8" s="1">
-        <v>6</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>24</v>
+        <v>16</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8" t="s">
+        <v>140</v>
+      </c>
+      <c r="F8" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D9" s="1">
+      <c r="D9">
         <v>7</v>
       </c>
       <c r="E9" t="s">
-        <v>29</v>
-      </c>
-      <c r="F9" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="F9" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D10" s="1">
-        <v>8</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>20</v>
+        <v>16</v>
+      </c>
+      <c r="D10">
+        <v>1</v>
+      </c>
+      <c r="E10" t="s">
+        <v>140</v>
+      </c>
+      <c r="F10" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D11" s="1">
-        <v>5</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>22</v>
+      <c r="D11">
+        <v>9</v>
+      </c>
+      <c r="E11" t="s">
+        <v>139</v>
+      </c>
+      <c r="F11" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D12" s="1">
-        <v>6</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>32</v>
+        <v>1</v>
+      </c>
+      <c r="E12" t="s">
+        <v>140</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>18</v>
       </c>
       <c r="D13" s="1">
+        <v>5</v>
+      </c>
+      <c r="E13" t="s">
+        <v>139</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14">
         <v>7</v>
       </c>
-      <c r="E13" s="1" t="s">
+      <c r="B14" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D14" s="1">
+        <v>1</v>
+      </c>
+      <c r="E14" t="s">
+        <v>140</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>7</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D15" s="1">
+        <v>6</v>
+      </c>
+      <c r="E15" t="s">
+        <v>139</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>8</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D16" s="1">
+        <v>1</v>
+      </c>
+      <c r="E16" t="s">
+        <v>140</v>
+      </c>
+      <c r="F16" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>8</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D17" s="1">
+        <v>7</v>
+      </c>
+      <c r="E17" t="s">
+        <v>139</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>9</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D18" s="1">
+        <v>1</v>
+      </c>
+      <c r="E18" t="s">
+        <v>140</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>9</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19" s="1">
+        <v>8</v>
+      </c>
+      <c r="E19" t="s">
+        <v>139</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>10</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D20" s="1">
+        <v>1</v>
+      </c>
+      <c r="E20" t="s">
+        <v>140</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>10</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D21" s="1">
+        <v>5</v>
+      </c>
+      <c r="E21" t="s">
+        <v>139</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>11</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D22" s="1">
+        <v>1</v>
+      </c>
+      <c r="E22" t="s">
+        <v>140</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>11</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D23" s="1">
+        <v>6</v>
+      </c>
+      <c r="E23" t="s">
+        <v>139</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>12</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D24" s="1">
+        <v>1</v>
+      </c>
+      <c r="E24" t="s">
+        <v>140</v>
+      </c>
+      <c r="F24" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="F13" s="1" t="s">
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>12</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D25" s="1">
+        <v>7</v>
+      </c>
+      <c r="E25" t="s">
+        <v>139</v>
+      </c>
+      <c r="F25" s="1" t="s">
         <v>26</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:F1 A13:D13 A2:D2 F2 A3:D3 F3 A4:D4 F4 A5:D5 F5 A6:D6 F6 A7:D7 F7 A8:D8 F8 A9:D9 F9 A10:D10 F10 A11:D11 F11 A12:D12 F12 F13" numberStoredAsText="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
 
@@ -1283,19 +1533,19 @@
       <c r="R1" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="S1" s="9" t="s">
+      <c r="S1" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="T1" s="9" t="s">
+      <c r="T1" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="U1" s="9" t="s">
+      <c r="U1" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="V1" s="9" t="s">
+      <c r="V1" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="W1" s="9" t="s">
+      <c r="W1" s="10" t="s">
         <v>27</v>
       </c>
     </row>
@@ -1570,7 +1820,7 @@
       <c r="S5" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="T5" s="4" t="s">
+      <c r="T5" s="9" t="s">
         <v>22</v>
       </c>
       <c r="U5" s="1" t="s">
@@ -1641,7 +1891,7 @@
       <c r="T6" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="U6" s="4" t="s">
+      <c r="U6" s="9" t="s">
         <v>24</v>
       </c>
       <c r="V6" s="1" t="s">
@@ -1712,7 +1962,7 @@
       <c r="U7" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="V7" s="4" t="s">
+      <c r="V7" s="9" t="s">
         <v>26</v>
       </c>
     </row>
@@ -1771,7 +2021,7 @@
       <c r="R8" s="1">
         <v>-2</v>
       </c>
-      <c r="S8" s="4" t="s">
+      <c r="S8" s="9" t="s">
         <v>20</v>
       </c>
       <c r="T8" s="1" t="s">
@@ -1851,7 +2101,7 @@
       <c r="V9" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="W9" s="4" t="s">
+      <c r="W9" s="9" t="s">
         <v>28</v>
       </c>
     </row>
@@ -1894,7 +2144,7 @@
       <c r="F1" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="G1" s="10" t="s">
         <v>29</v>
       </c>
     </row>
@@ -2113,16 +2363,16 @@
       <c r="D1" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="E1" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="F1" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="G1" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="H1" s="9" t="s">
+      <c r="H1" s="10" t="s">
         <v>33</v>
       </c>
       <c r="I1" s="2" t="s">

</xml_diff>

<commit_message>
add library_variable_codelist_value (submission value) to results
</commit_message>
<xml_diff>
--- a/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
+++ b/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10920"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rich/Documents/github/core-contributor/rules/NEW-RULE/negative/01/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BD11A63-9B06-A04F-AC9C-415339A9B030}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFD94C61-1069-864E-82E5-357FE83C94A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2520" yWindow="1100" windowWidth="30240" windowHeight="18980" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="36420" yWindow="-1180" windowWidth="30240" windowHeight="18980" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="119">
   <si>
     <t>Product</t>
   </si>
@@ -371,6 +371,15 @@
   </si>
   <si>
     <t>Outcome of Event</t>
+  </si>
+  <si>
+    <t>library_variable_codelist_value</t>
+  </si>
+  <si>
+    <t>OUT</t>
+  </si>
+  <si>
+    <t>NY</t>
   </si>
 </sst>
 </file>
@@ -845,7 +854,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="5" max="5" width="18.5" bestFit="1" customWidth="1"/>
@@ -952,8 +961,8 @@
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A6" s="1">
-        <v>2</v>
+      <c r="A6" s="5">
+        <v>1</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>6</v>
@@ -962,13 +971,13 @@
         <v>12</v>
       </c>
       <c r="D6" s="5">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>105</v>
+        <v>116</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
@@ -985,10 +994,10 @@
         <v>6</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>91</v>
+        <v>44</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
@@ -1005,55 +1014,55 @@
         <v>6</v>
       </c>
       <c r="E8" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A9" s="1">
+        <v>2</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D9" s="5">
+        <v>6</v>
+      </c>
+      <c r="E9" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="F8" s="5" t="s">
+      <c r="F9" s="5" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A9" s="5">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A10" s="5">
         <v>2</v>
       </c>
-      <c r="B9" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="D9" s="5">
-        <v>6</v>
-      </c>
-      <c r="E9" s="5" t="s">
+      <c r="B10" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D10" s="5">
+        <v>6</v>
+      </c>
+      <c r="E10" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="F9" s="5" t="s">
+      <c r="F10" s="5" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A10" s="1">
-        <v>3</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="D10" s="5">
-        <v>8</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>45</v>
-      </c>
-    </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A11" s="1">
-        <v>3</v>
+      <c r="A11" s="5">
+        <v>2</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>6</v>
@@ -1062,13 +1071,13 @@
         <v>12</v>
       </c>
       <c r="D11" s="5">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>106</v>
+        <v>116</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
@@ -1085,14 +1094,14 @@
         <v>8</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>109</v>
+        <v>45</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A13" s="5">
+      <c r="A13" s="1">
         <v>3</v>
       </c>
       <c r="B13" s="1" t="s">
@@ -1105,15 +1114,15 @@
         <v>8</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>6</v>
@@ -1122,18 +1131,18 @@
         <v>12</v>
       </c>
       <c r="D14" s="5">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>41</v>
+        <v>109</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A15" s="1">
-        <v>4</v>
+      <c r="A15" s="5">
+        <v>3</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>6</v>
@@ -1142,18 +1151,18 @@
         <v>12</v>
       </c>
       <c r="D15" s="5">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>104</v>
+        <v>114</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A16" s="1">
-        <v>4</v>
+      <c r="A16" s="5">
+        <v>3</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>6</v>
@@ -1162,17 +1171,17 @@
         <v>12</v>
       </c>
       <c r="D16" s="5">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>109</v>
+        <v>118</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A17" s="5">
+      <c r="A17" s="1">
         <v>4</v>
       </c>
       <c r="B17" s="1" t="s">
@@ -1185,15 +1194,15 @@
         <v>9</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>114</v>
+        <v>41</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>6</v>
@@ -1202,18 +1211,18 @@
         <v>12</v>
       </c>
       <c r="D18" s="5">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>45</v>
+        <v>104</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>6</v>
@@ -1222,18 +1231,18 @@
         <v>12</v>
       </c>
       <c r="D19" s="5">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="F19" s="5">
-        <v>77</v>
+        <v>107</v>
+      </c>
+      <c r="F19" s="5" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A20" s="1">
-        <v>5</v>
+      <c r="A20" s="5">
+        <v>4</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>6</v>
@@ -1242,33 +1251,133 @@
         <v>12</v>
       </c>
       <c r="D20" s="5">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" s="5">
+        <v>4</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D21" s="5">
         <v>5</v>
       </c>
-      <c r="B21" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C21" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="D21" s="5">
+      <c r="E21" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="F21" s="5" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A22" s="1">
+        <v>5</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D22" s="5">
         <v>10</v>
       </c>
-      <c r="E21" s="5" t="s">
+      <c r="E22" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="F22" s="5" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A23" s="1">
+        <v>5</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D23" s="5">
+        <v>10</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="F23" s="5">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A24" s="1">
+        <v>5</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D24" s="5">
+        <v>10</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="F24" s="5" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A25" s="5">
+        <v>5</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D25" s="5">
+        <v>10</v>
+      </c>
+      <c r="E25" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="F21" s="5" t="s">
+      <c r="F25" s="5" t="s">
         <v>114</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A26" s="5">
+        <v>5</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D26" s="5">
+        <v>5</v>
+      </c>
+      <c r="E26" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="F26" s="5" t="s">
+        <v>118</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated rule but not yet ready for review
</commit_message>
<xml_diff>
--- a/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
+++ b/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
@@ -36,7 +36,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -52,7 +52,18 @@
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
+      <color rgb="FF000000"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
       <b/>
+      <color rgb="FF000000"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <i/>
       <color rgb="FF000000"/>
     </font>
     <font>
@@ -72,7 +83,7 @@
       <color rgb="FF000000"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none">
         <bgColor/>
@@ -86,6 +97,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFCC"/>
+        <bgColor/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor/>
       </patternFill>
     </fill>
@@ -115,15 +138,17 @@
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -509,7 +534,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F7"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -548,7 +573,7 @@
         <v>FATEST</v>
       </c>
       <c r="F2" s="2" t="str">
-        <v>Epoch</v>
+        <v>Toxicity Grade</v>
       </c>
     </row>
     <row r="3">
@@ -568,288 +593,474 @@
         <v>FATESTCD</v>
       </c>
       <c r="F3" s="2" t="str">
-        <v>EPOCH</v>
+        <v>TOXGRD</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2">
+        <v>2</v>
+      </c>
+      <c r="B4" s="2" t="str">
+        <v>fa.xpt</v>
+      </c>
+      <c r="C4" s="2" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D4" s="2">
+        <v>6</v>
+      </c>
+      <c r="E4" s="2" t="str">
+        <v>FATEST</v>
+      </c>
+      <c r="F4" s="4" t="str">
+        <v>Occurence Indicator</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2">
+        <v>2</v>
+      </c>
+      <c r="B5" s="2" t="str">
+        <v>fa.xpt</v>
+      </c>
+      <c r="C5" s="2" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D5" s="2">
+        <v>6</v>
+      </c>
+      <c r="E5" s="2" t="str">
+        <v>FATESTCD</v>
+      </c>
+      <c r="F5" s="4" t="str">
+        <v>OCCURS</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2">
+        <v>3</v>
+      </c>
+      <c r="B6" s="2" t="str">
+        <v>fa.xpt</v>
+      </c>
+      <c r="C6" s="2" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D6" s="2">
+        <v>7</v>
+      </c>
+      <c r="E6" s="2" t="str">
+        <v>FATEST</v>
+      </c>
+      <c r="F6" s="4" t="str">
+        <v>Anatomical Region of Specimen</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2">
+        <v>3</v>
+      </c>
+      <c r="B7" s="2" t="str">
+        <v>fa.xpt</v>
+      </c>
+      <c r="C7" s="2" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D7" s="2">
+        <v>7</v>
+      </c>
+      <c r="E7" s="2" t="str">
+        <v>FATESTCD</v>
+      </c>
+      <c r="F7" s="4" t="str">
+        <v>BSORRES</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F7"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q5"/>
+  <dimension ref="A1:Q7"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="str">
+      <c r="A1" s="5" t="str">
         <v>STUDYID</v>
       </c>
-      <c r="B1" s="4" t="str">
+      <c r="B1" s="5" t="str">
         <v>DOMAIN</v>
       </c>
-      <c r="C1" s="4" t="str">
+      <c r="C1" s="5" t="str">
         <v>USUBJID</v>
       </c>
-      <c r="D1" s="4" t="str">
+      <c r="D1" s="5" t="str">
         <v>FASEQ</v>
       </c>
-      <c r="E1" s="4" t="str">
+      <c r="E1" s="5" t="str">
         <v>FAGRPID</v>
       </c>
-      <c r="F1" s="4" t="str">
+      <c r="F1" s="5" t="str">
         <v>FATESTCD</v>
       </c>
-      <c r="G1" s="4" t="str">
+      <c r="G1" s="5" t="str">
         <v>FATEST</v>
       </c>
-      <c r="H1" s="4" t="str">
+      <c r="H1" s="5" t="str">
         <v>FAOBJ</v>
       </c>
-      <c r="I1" s="4" t="str">
+      <c r="I1" s="5" t="str">
         <v>FADECOD</v>
       </c>
-      <c r="J1" s="4" t="str">
+      <c r="J1" s="5" t="str">
         <v>FACAT</v>
       </c>
-      <c r="K1" s="4" t="str">
+      <c r="K1" s="5" t="str">
         <v>FAORRES</v>
       </c>
-      <c r="L1" s="4" t="str">
+      <c r="L1" s="5" t="str">
         <v>FASTRESC</v>
       </c>
-      <c r="M1" s="4" t="str">
+      <c r="M1" s="5" t="str">
         <v>FALOC</v>
       </c>
-      <c r="N1" s="4" t="str">
+      <c r="N1" s="5" t="str">
         <v>VISITNUM</v>
       </c>
-      <c r="O1" s="4" t="str">
+      <c r="O1" s="5" t="str">
         <v>EPOCH</v>
       </c>
-      <c r="P1" s="4" t="str">
+      <c r="P1" s="5" t="str">
         <v>FADTC</v>
       </c>
-      <c r="Q1" s="4" t="str">
+      <c r="Q1" s="5" t="str">
         <v>FADY</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="str">
+      <c r="A2" s="6" t="str">
         <v>Study Identifier</v>
       </c>
-      <c r="B2" s="5" t="str">
+      <c r="B2" s="7" t="str">
         <v>Domain Abbreviation</v>
       </c>
-      <c r="C2" s="5" t="str">
+      <c r="C2" s="7" t="str">
         <v>Unique Subject Identifier</v>
       </c>
-      <c r="D2" s="5" t="str">
+      <c r="D2" s="7" t="str">
         <v>Sequence Number</v>
       </c>
-      <c r="E2" s="5" t="str">
+      <c r="E2" s="7" t="str">
         <v>Group ID</v>
       </c>
-      <c r="F2" s="5" t="str">
+      <c r="F2" s="7" t="str">
         <v>Findings About Test Short Name</v>
       </c>
-      <c r="G2" s="5" t="str">
+      <c r="G2" s="7" t="str">
         <v>Findings About Test Name</v>
       </c>
-      <c r="H2" s="5" t="str">
+      <c r="H2" s="7" t="str">
         <v>Object of the Observation</v>
       </c>
-      <c r="I2" s="5" t="str">
+      <c r="I2" s="7" t="str">
         <v>Dictionary-Derived Term</v>
       </c>
-      <c r="J2" s="5" t="str">
+      <c r="J2" s="7" t="str">
         <v>Category for Findings About</v>
       </c>
-      <c r="K2" s="5" t="str">
+      <c r="K2" s="7" t="str">
         <v>Result or Finding in Original Units</v>
       </c>
-      <c r="L2" s="5" t="str">
+      <c r="L2" s="7" t="str">
         <v>Character Result/Finding in Std Format</v>
       </c>
-      <c r="M2" s="5" t="str">
+      <c r="M2" s="7" t="str">
         <v>Location of the Finding About</v>
       </c>
-      <c r="N2" s="5" t="str">
+      <c r="N2" s="7" t="str">
         <v>Visit Number</v>
       </c>
-      <c r="O2" s="5" t="str">
+      <c r="O2" s="7" t="str">
         <v>Epoch</v>
       </c>
-      <c r="P2" s="5" t="str">
+      <c r="P2" s="7" t="str">
         <v>Date/Time of Collection</v>
       </c>
-      <c r="Q2" s="5" t="str">
+      <c r="Q2" s="7" t="str">
         <v>Study Day of Collection</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="B3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="C3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="D3" s="5" t="str">
+      <c r="A3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="B3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="C3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="D3" s="7" t="str">
         <v>Num</v>
       </c>
-      <c r="E3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="F3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="G3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="H3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="I3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="J3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="K3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="L3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="M3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="N3" s="5" t="str">
+      <c r="E3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="F3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="G3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="H3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="I3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="J3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="K3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="L3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="M3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="N3" s="7" t="str">
         <v>Num</v>
       </c>
-      <c r="O3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="P3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="Q3" s="5" t="str">
+      <c r="O3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="P3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="Q3" s="7" t="str">
         <v>Num</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="B4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="C4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="D4" s="5" t="str">
+      <c r="A4" s="7" t="str">
+        <v>50</v>
+      </c>
+      <c r="B4" s="7" t="str">
+        <v>50</v>
+      </c>
+      <c r="C4" s="7" t="str">
+        <v>50</v>
+      </c>
+      <c r="D4" s="7" t="str">
         <v>8</v>
       </c>
-      <c r="E4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="F4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="G4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="H4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="I4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="J4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="K4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="L4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="M4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="N4" s="5" t="str">
+      <c r="E4" s="7" t="str">
+        <v>50</v>
+      </c>
+      <c r="F4" s="7" t="str">
+        <v>50</v>
+      </c>
+      <c r="G4" s="7" t="str">
+        <v>50</v>
+      </c>
+      <c r="H4" s="7" t="str">
+        <v>50</v>
+      </c>
+      <c r="I4" s="7" t="str">
+        <v>50</v>
+      </c>
+      <c r="J4" s="7" t="str">
+        <v>50</v>
+      </c>
+      <c r="K4" s="7" t="str">
+        <v>50</v>
+      </c>
+      <c r="L4" s="7" t="str">
+        <v>50</v>
+      </c>
+      <c r="M4" s="7" t="str">
+        <v>50</v>
+      </c>
+      <c r="N4" s="7" t="str">
         <v>8</v>
       </c>
-      <c r="O4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="P4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="Q4" s="5" t="str">
+      <c r="O4" s="7" t="str">
+        <v>50</v>
+      </c>
+      <c r="P4" s="7" t="str">
+        <v>50</v>
+      </c>
+      <c r="Q4" s="7" t="str">
         <v>8</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="str">
+      <c r="A5" s="4" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B5" s="6" t="str">
+      <c r="B5" s="4" t="str">
         <v>FA</v>
       </c>
-      <c r="C5" s="6" t="str">
+      <c r="C5" s="4" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D5" s="6">
+      <c r="D5" s="4">
         <v>1</v>
       </c>
-      <c r="E5" s="6">
+      <c r="E5" s="4">
         <v>1</v>
       </c>
-      <c r="F5" s="7" t="str">
-        <v>EPOCH</v>
-      </c>
-      <c r="G5" s="7" t="str">
-        <v>Epoch</v>
-      </c>
-      <c r="H5" s="6" t="str">
+      <c r="F5" s="8" t="str">
+        <v>TOXGRD</v>
+      </c>
+      <c r="G5" s="9" t="str">
+        <v>Toxicity Grade</v>
+      </c>
+      <c r="H5" s="4" t="str">
         <v>ERYTHEMA</v>
       </c>
-      <c r="I5" s="6" t="str">
+      <c r="I5" s="4" t="str">
         <v/>
       </c>
-      <c r="J5" s="6" t="str">
+      <c r="J5" s="4" t="str">
         <v>INJECTION SITE REACTION</v>
       </c>
-      <c r="K5" s="6" t="str">
+      <c r="K5" s="4" t="str">
         <v>MODERATE</v>
       </c>
-      <c r="L5" s="6" t="str">
+      <c r="L5" s="4" t="str">
         <v>MODERATE</v>
       </c>
-      <c r="M5" s="6" t="str">
+      <c r="M5" s="4" t="str">
         <v>ARM</v>
       </c>
-      <c r="N5" s="6" t="str">
+      <c r="N5" s="4" t="str">
         <v/>
       </c>
-      <c r="O5" s="6" t="str">
+      <c r="O5" s="4" t="str">
         <v>TREATMENT</v>
       </c>
-      <c r="P5" s="6" t="str">
+      <c r="P5" s="4" t="str">
         <v>2012-12-02</v>
       </c>
-      <c r="Q5" s="6">
+      <c r="Q5" s="4">
         <v>3</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="str">
+        <v>CDISCPILOT01</v>
+      </c>
+      <c r="B6" s="4" t="str">
+        <v>FA</v>
+      </c>
+      <c r="C6" s="4" t="str">
+        <v>CDISC002</v>
+      </c>
+      <c r="D6" s="4">
+        <v>1</v>
+      </c>
+      <c r="E6" s="4">
+        <v>1</v>
+      </c>
+      <c r="F6" s="9" t="str">
+        <v>OCCURS</v>
+      </c>
+      <c r="G6" s="9" t="str">
+        <v>Occurence Indicator</v>
+      </c>
+      <c r="H6" s="4" t="str">
+        <v>ERYTHEMA</v>
+      </c>
+      <c r="I6" s="4" t="str">
+        <v/>
+      </c>
+      <c r="J6" s="4" t="str">
+        <v>INJECTION SITE REACTION</v>
+      </c>
+      <c r="K6" s="4" t="str">
+        <v>MODERATE</v>
+      </c>
+      <c r="L6" s="4" t="str">
+        <v>MODERATE</v>
+      </c>
+      <c r="M6" s="4" t="str">
+        <v>ARM</v>
+      </c>
+      <c r="N6" s="4" t="str">
+        <v/>
+      </c>
+      <c r="O6" s="4" t="str">
+        <v>TREATMENT</v>
+      </c>
+      <c r="P6" s="4" t="str">
+        <v>2012-12-03</v>
+      </c>
+      <c r="Q6" s="4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="str">
+        <v>CDISCPILOT01</v>
+      </c>
+      <c r="B7" s="4" t="str">
+        <v>FA</v>
+      </c>
+      <c r="C7" s="4" t="str">
+        <v>CDISC003</v>
+      </c>
+      <c r="D7" s="4">
+        <v>1</v>
+      </c>
+      <c r="E7" s="4">
+        <v>1</v>
+      </c>
+      <c r="F7" s="9" t="str">
+        <v>BSORRES</v>
+      </c>
+      <c r="G7" s="9" t="str">
+        <v>Anatomical Region of Specimen</v>
+      </c>
+      <c r="H7" s="4" t="str">
+        <v>ERYTHEMA</v>
+      </c>
+      <c r="I7" s="4" t="str">
+        <v/>
+      </c>
+      <c r="J7" s="4" t="str">
+        <v>INJECTION SITE REACTION</v>
+      </c>
+      <c r="K7" s="4" t="str">
+        <v>MODERATE</v>
+      </c>
+      <c r="L7" s="4" t="str">
+        <v>MODERATE</v>
+      </c>
+      <c r="M7" s="4" t="str">
+        <v>ARM</v>
+      </c>
+      <c r="N7" s="4" t="str">
+        <v/>
+      </c>
+      <c r="O7" s="4" t="str">
+        <v>TREATMENT</v>
+      </c>
+      <c r="P7" s="4" t="str">
+        <v>2012-12-04</v>
+      </c>
+      <c r="Q7" s="4">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Q5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
CG0011 create: part B updated rule logic and test data - to check further for interval
</commit_message>
<xml_diff>
--- a/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
+++ b/rules/NEW-RULE/negative/01/data/new-rule-negative-01.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marisa_wyckmans\CORE\CDISC_Rule_Authoring\core-contributor\rules\NEW-RULE\negative\01\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7FF63A0-4386-40F0-9EAB-9EAB2A34646E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC4CCCA9-5DEB-4864-BEC3-3CD88D1E1064}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="21240" windowHeight="15270" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,20 @@
     <sheet name="Validation" sheetId="3" r:id="rId3"/>
     <sheet name="qs.xpt" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -333,7 +346,7 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>

</xml_diff>